<commit_message>
transformacion a csv, edicion
</commit_message>
<xml_diff>
--- a/estadistica2/data/velasquez_faure.xlsx
+++ b/estadistica2/data/velasquez_faure.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10329"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kennethbunker/Library/CloudStorage/Dropbox/GitHub/uss/estadistica2/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41300B40-7A70-8147-972B-6ADABDC002C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B78D78C6-8C74-EB4B-B732-38ECA218ADF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,6 +17,7 @@
     <sheet name="codebook" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">codebook!$A$1:$E$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">data!$A$1:$I$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="33">
   <si>
     <t>country_name</t>
   </si>
@@ -119,6 +120,21 @@
   </si>
   <si>
     <t>ethnic</t>
+  </si>
+  <si>
+    <t>variable</t>
+  </si>
+  <si>
+    <t>descripcion</t>
+  </si>
+  <si>
+    <t>medicion</t>
+  </si>
+  <si>
+    <t>min</t>
+  </si>
+  <si>
+    <t>max</t>
   </si>
 </sst>
 </file>
@@ -632,7 +648,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
@@ -641,6 +657,8 @@
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="37" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1000,6 +1018,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="10.83203125" customWidth="1"/>
     <col min="6" max="6" width="11.5" style="4"/>
     <col min="7" max="7" width="11.5" style="2"/>
@@ -6799,9 +6818,86 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1BBE8D6-39CA-7F44-81E8-2B0BB2DB2329}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" s="8" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E1" xr:uid="{D1BBE8D6-39CA-7F44-81E8-2B0BB2DB2329}"/>
+  <conditionalFormatting sqref="A2">
+    <cfRule type="duplicateValues" priority="1"/>
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>